<commit_message>
Update Excel practice files and READMEs
</commit_message>
<xml_diff>
--- a/Excel/05_Cell_Formats/Pinterest_Cell_Formats_Practice.xlsx.xlsx
+++ b/Excel/05_Cell_Formats/Pinterest_Cell_Formats_Practice.xlsx.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/afea116efc88aa0e/Desktop/Pinterest-Analytics-Project/Excel/05_Cell_Formats/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="142" documentId="8_{CEDE7376-32D0-4D72-A38D-540EC3D7BDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD0004EA-6267-41DB-9D95-383D22BA0352}"/>
+  <xr:revisionPtr revIDLastSave="144" documentId="8_{CEDE7376-32D0-4D72-A38D-540EC3D7BDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ACC3D63E-52D6-4335-858F-D3A04DF3294D}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{14F6D59A-929E-4E3A-B68A-E346893EE24F}"/>
   </bookViews>
@@ -781,11 +781,11 @@
   <dimension ref="A1:I20"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="25.54296875" style="2" customWidth="1"/>
-    <col min="2" max="3" width="25.54296875" style="5" customWidth="1"/>
-    <col min="4" max="7" width="25.54296875" style="3" customWidth="1"/>
-    <col min="8" max="8" width="25.54296875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="25.54296875" style="4" customWidth="1"/>
+    <col min="1" max="1" width="34.08984375" style="2" customWidth="1"/>
+    <col min="2" max="3" width="34.08984375" style="5" customWidth="1"/>
+    <col min="4" max="7" width="34.08984375" style="3" customWidth="1"/>
+    <col min="8" max="8" width="34.08984375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="34.08984375" style="4" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="54" customHeight="1" x14ac:dyDescent="0.35">
@@ -817,7 +817,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="44" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" ht="58" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="6">
         <v>46266</v>
       </c>

</xml_diff>